<commit_message>
Fix March 2026 billing showing 0 for 14 employees
Formula cells (=2000+213 etc.) in Clients- March26 sheet were
returning None via data_only after previous openpyxl save cleared
Excel's formula cache. Evaluated all 14 formulas to plain numbers.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/uploads/TR Billing V_S Cost Analysis - March.xlsx
+++ b/uploads/TR Billing V_S Cost Analysis - March.xlsx
@@ -51856,9 +51856,8 @@
           <t>Chintan</t>
         </is>
       </c>
-      <c r="E10" s="52">
-        <f>200+688</f>
-        <v/>
+      <c r="E10" s="52" t="n">
+        <v>888</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -51876,9 +51875,8 @@
           <t>Purnayu</t>
         </is>
       </c>
-      <c r="E11" s="52">
-        <f>200+688</f>
-        <v/>
+      <c r="E11" s="52" t="n">
+        <v>888</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
@@ -51896,9 +51894,8 @@
           <t>Abhay Panchal</t>
         </is>
       </c>
-      <c r="E12" s="52">
-        <f>200+688</f>
-        <v/>
+      <c r="E12" s="52" t="n">
+        <v>888</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
@@ -51935,9 +51932,8 @@
           <t>Jerry John Murphy</t>
         </is>
       </c>
-      <c r="E14" s="52">
-        <f>2090.91+25</f>
-        <v/>
+      <c r="E14" s="52" t="n">
+        <v>2115.91</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
@@ -52088,9 +52084,8 @@
           <t>Rochelle Extross</t>
         </is>
       </c>
-      <c r="E22" s="52">
-        <f>2000+213</f>
-        <v/>
+      <c r="E22" s="52" t="n">
+        <v>2213</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
@@ -52108,9 +52103,8 @@
           <t xml:space="preserve">Mudassar </t>
         </is>
       </c>
-      <c r="E23" s="52">
-        <f>2100+213</f>
-        <v/>
+      <c r="E23" s="52" t="n">
+        <v>2313</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
@@ -52128,9 +52122,8 @@
           <t>Pooja Kumari</t>
         </is>
       </c>
-      <c r="E24" s="52">
-        <f>2100+213</f>
-        <v/>
+      <c r="E24" s="52" t="n">
+        <v>2313</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
@@ -52148,9 +52141,8 @@
           <t>Vishal Patel</t>
         </is>
       </c>
-      <c r="E25" s="52">
-        <f>2100+213</f>
-        <v/>
+      <c r="E25" s="52" t="n">
+        <v>2313</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
@@ -52168,9 +52160,8 @@
           <t>Viraj</t>
         </is>
       </c>
-      <c r="E26" s="52">
-        <f>1909.09+213</f>
-        <v/>
+      <c r="E26" s="52" t="n">
+        <v>2122.09</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
@@ -52188,9 +52179,8 @@
           <t>Ashok</t>
         </is>
       </c>
-      <c r="E27" s="52">
-        <f>2000+213</f>
-        <v/>
+      <c r="E27" s="52" t="n">
+        <v>2213</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
@@ -52208,9 +52198,8 @@
           <t>Madhuri</t>
         </is>
       </c>
-      <c r="E28" s="52">
-        <f>1727.27+213</f>
-        <v/>
+      <c r="E28" s="52" t="n">
+        <v>1940.27</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
@@ -52481,9 +52470,8 @@
           <t>Vinodh K</t>
         </is>
       </c>
-      <c r="E44" s="6">
-        <f>4900-578</f>
-        <v/>
+      <c r="E44" s="6" t="n">
+        <v>4322</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
@@ -52497,9 +52485,8 @@
           <t>Amritha</t>
         </is>
       </c>
-      <c r="E45" s="6">
-        <f>6482-578</f>
-        <v/>
+      <c r="E45" s="6" t="n">
+        <v>5904</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
@@ -52513,9 +52500,8 @@
           <t>Kimaya</t>
         </is>
       </c>
-      <c r="E46" s="6">
-        <f>5100-579</f>
-        <v/>
+      <c r="E46" s="6" t="n">
+        <v>4521</v>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">

</xml_diff>